<commit_message>
edited test cases and display
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-42_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-42_Test_Cases.xlsx
@@ -23,7 +23,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC14" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC15" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC16" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC17" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -463,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -919,7 +918,7 @@
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>A booking can only be requested once the event is Approved or in Planning (team decision)</t>
+          <t>A venue cannot be requested for a completed, cancelled or rejected event (existing SPM-47 rule)</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1034,94 +1033,62 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>TC17</t>
-        </is>
-      </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>SPM-42-TC17</t>
-        </is>
-      </c>
-      <c r="C20" s="11" t="inlineStr">
-        <is>
-          <t>An event or session with an active request cannot request a second venue (#109)</t>
-        </is>
-      </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>AC4, AC5</t>
-        </is>
-      </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="F20" s="11" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>AC</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Acceptance Criterion</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Covered by</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="n"/>
+    </row>
+    <row r="23" ht="44.5" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>AC1</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>The Event Coordinator can select a suitable venue.</t>
         </is>
       </c>
       <c r="C23" s="8" t="n"/>
       <c r="D23" s="9" t="n"/>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>Covered by</t>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>SPM-42-TC01
+SPM-42-TC02
+SPM-42-TC12</t>
         </is>
       </c>
       <c r="F23" s="9" t="n"/>
     </row>
-    <row r="24" ht="44.5" customHeight="1">
+    <row r="24" ht="125.5" customHeight="1">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>AC1</t>
+          <t>AC2</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>The Event Coordinator can select a suitable venue.</t>
+          <t>The request specifies one or more of the venue's fixed AM, PM or Night slots for the required date; an event spanning multiple slots consumes each of them in full.</t>
         </is>
       </c>
       <c r="C24" s="8" t="n"/>
       <c r="D24" s="9" t="n"/>
       <c r="E24" s="11" t="inlineStr">
-        <is>
-          <t>SPM-42-TC01
-SPM-42-TC02
-SPM-42-TC12</t>
-        </is>
-      </c>
-      <c r="F24" s="9" t="n"/>
-    </row>
-    <row r="25" ht="125.5" customHeight="1">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>AC2</t>
-        </is>
-      </c>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>The request specifies one or more of the venue's fixed AM, PM or Night slots for the required date; an event spanning multiple slots consumes each of them in full.</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="9" t="n"/>
-      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>SPM-42-TC03
 SPM-42-TC04
@@ -1134,22 +1101,22 @@
 SPM-42-TC16</t>
         </is>
       </c>
-      <c r="F25" s="9" t="n"/>
-    </row>
-    <row r="26" ht="58" customHeight="1">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="F24" s="9" t="n"/>
+    </row>
+    <row r="25" ht="58" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>AC3</t>
         </is>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>Where setup or turnaround time is required, the immediately adjacent slot (before the event for setup, after for turnaround, including the previous or following day where applicable) is included in the request.</t>
         </is>
       </c>
-      <c r="C26" s="8" t="n"/>
-      <c r="D26" s="9" t="n"/>
-      <c r="E26" s="11" t="inlineStr">
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="9" t="n"/>
+      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>SPM-42-TC06
 SPM-42-TC07
@@ -1157,123 +1124,121 @@
 SPM-42-TC16</t>
         </is>
       </c>
+      <c r="F25" s="9" t="n"/>
+    </row>
+    <row r="26" ht="44.5" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>AC4</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>For a multi-session event, a booking request is made per session, using that session's own date, time and requirements rather than the event's.</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="n"/>
+      <c r="D26" s="9" t="n"/>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>SPM-42-TC04
+SPM-42-TC08
+SPM-42-TC09</t>
+        </is>
+      </c>
       <c r="F26" s="9" t="n"/>
     </row>
-    <row r="27" ht="58" customHeight="1">
+    <row r="27" ht="31" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>AC4</t>
+          <t>AC5</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>For a multi-session event, a booking request is made per session, using that session's own date, time and requirements rather than the event's.</t>
+          <t>The request is associated with the relevant event (and session, where applicable).</t>
         </is>
       </c>
       <c r="C27" s="8" t="n"/>
       <c r="D27" s="9" t="n"/>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>SPM-42-TC04
-SPM-42-TC08
-SPM-42-TC09
-SPM-42-TC17</t>
+          <t>SPM-42-TC09
+SPM-42-TC10</t>
         </is>
       </c>
       <c r="F27" s="9" t="n"/>
     </row>
-    <row r="28" ht="44.5" customHeight="1">
+    <row r="28" ht="31" customHeight="1">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>AC5</t>
+          <t>AC6</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>The request is associated with the relevant event (and session, where applicable).</t>
+          <t>Venue requirements are included in the request.</t>
         </is>
       </c>
       <c r="C28" s="8" t="n"/>
       <c r="D28" s="9" t="n"/>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>SPM-42-TC09
-SPM-42-TC10
-SPM-42-TC17</t>
+          <t>SPM-42-TC01
+SPM-42-TC03</t>
         </is>
       </c>
       <c r="F28" s="9" t="n"/>
     </row>
-    <row r="29" ht="31" customHeight="1">
+    <row r="29" ht="44.5" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>AC6</t>
+          <t>AC7</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>Venue requirements are included in the request.</t>
+          <t>The request is submitted to Venue Staff for review.</t>
         </is>
       </c>
       <c r="C29" s="8" t="n"/>
       <c r="D29" s="9" t="n"/>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>SPM-42-TC01
-SPM-42-TC03</t>
+          <t>SPM-42-TC11
+SPM-42-TC12
+SPM-42-TC13</t>
         </is>
       </c>
       <c r="F29" s="9" t="n"/>
     </row>
-    <row r="30" ht="44.5" customHeight="1">
+    <row r="30" ht="17.5" customHeight="1">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>AC7</t>
+          <t>AC8</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>The request is submitted to Venue Staff for review.</t>
+          <t>The venue booking request has a pending status.</t>
         </is>
       </c>
       <c r="C30" s="8" t="n"/>
       <c r="D30" s="9" t="n"/>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>SPM-42-TC11
-SPM-42-TC12
-SPM-42-TC13</t>
+          <t>SPM-42-TC11</t>
         </is>
       </c>
       <c r="F30" s="9" t="n"/>
     </row>
-    <row r="31" ht="17.5" customHeight="1">
-      <c r="A31" s="11" t="inlineStr">
-        <is>
-          <t>AC8</t>
-        </is>
-      </c>
-      <c r="B31" s="11" t="inlineStr">
-        <is>
-          <t>The venue booking request has a pending status.</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="n"/>
-      <c r="D31" s="9" t="n"/>
-      <c r="E31" s="11" t="inlineStr">
-        <is>
-          <t>SPM-42-TC11</t>
-        </is>
-      </c>
-      <c r="F31" s="9" t="n"/>
-    </row>
-    <row r="33" ht="166" customHeight="1">
-      <c r="A33" s="7" t="inlineStr">
+    <row r="32" ht="166" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>Code reviewed</t>
         </is>
       </c>
-      <c r="B33" s="11" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>src/lib/venueBookingRequest.ts
 src/lib/__tests__/venueBookingRequest.test.ts
@@ -1289,10 +1254,10 @@
 docs/CUSTOMER_CLARIFICATIONS.md</t>
         </is>
       </c>
-      <c r="C33" s="8" t="n"/>
-      <c r="D33" s="8" t="n"/>
-      <c r="E33" s="8" t="n"/>
-      <c r="F33" s="9" t="n"/>
+      <c r="C32" s="8" t="n"/>
+      <c r="D32" s="8" t="n"/>
+      <c r="E32" s="8" t="n"/>
+      <c r="F32" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="20">
@@ -1305,17 +1270,17 @@
     <mergeCell ref="E28:F28"/>
     <mergeCell ref="B30:D30"/>
     <mergeCell ref="B1:F1"/>
-    <mergeCell ref="E31:F31"/>
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="E30:F30"/>
     <mergeCell ref="B26:D26"/>
     <mergeCell ref="E27:F27"/>
     <mergeCell ref="E26:F26"/>
     <mergeCell ref="B25:D25"/>
-    <mergeCell ref="B31:D31"/>
     <mergeCell ref="E25:F25"/>
-    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="B22:D22"/>
     <mergeCell ref="B27:D27"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="B32:F32"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
@@ -1334,7 +1299,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId17"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1373,7 +1337,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="112" customHeight="1">
+    <row r="3" ht="125.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1381,12 +1345,12 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm42.
-Logged in as Daniel Tan, assigned to spm42_three_sessions 'SPM42 Three-Session Forum' (status Approved; opening the Venue tab moves it to Planning, SPM-40). Sessions: 'Day 1' 1 Mar 2027 (2026-09-26 + 156) 09:00-12:00, expects 80, Theatre; 'Day 2' 2 Mar 2027 (2026-09-26 + 157) 14:00-17:00, expects 30, Classroom; 'Day 3' 3 Mar 2027 (2026-09-26 + 158) 19:00-22:00, expects 60, Banquet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="166" customHeight="1">
+          <t>npm run fixtures:spm42 has been run once at the start of this test pass (do not re-run it between cases - later cases use requests made in earlier ones).
+Logged in as Daniel Tan, assigned to spm42_three_sessions 'SPM42 Three-Session Forum' (status Approved). Sessions: 'Day 1' 1 Mar 2027 (2026-09-26 + 156) 09:00-12:00, expects 80, Theatre; 'Day 2' 2 Mar 2027 (2026-09-26 + 157) 14:00-17:00, expects 30, Classroom; 'Day 3' 3 Mar 2027 (2026-09-26 + 158) 19:00-22:00, expects 60, Banquet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="287.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1394,12 +1358,20 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Open the event 'SPM42 Three-Session Forum'
-2. Open the Venue tab (Find a venue)
-3. Choose Session 'Day 1', click 'Request booking' on 'Orchard Seminar Room (ORC-SEM)', check the date and slot shown, click 'Submit request'
-4. Choose Session 'Day 2', click 'Request booking' on 'Orchard Studio (ORC-STU)', check the date and slot shown, click 'Submit request'
-5. Choose Session 'Day 3', click 'Request booking' on 'Orchard Gallery (ORC-GAL)', check the date and slot shown, click 'Submit request'
-6. Look at the event's booking requests</t>
+          <t>1. Log in as daniel.tan@connectsphere.com / password123
+2. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
+3. Click 'SPM42 Three-Session Forum' in the list
+4. Click the 'Venue' tab
+5. In the 'Session' drop-down, choose 'Day 1'
+6. Find 'Orchard Seminar Room (ORC-SEM)' in the venue list and click its 'Request booking' button
+7. Check the Session, Date, ticked slot and Layout shown, then click 'Submit request' and click 'Back to Venue'
+8. In the 'Session' drop-down, choose 'Day 2'
+9. Find 'Orchard Studio (ORC-STU)' in the venue list and click its 'Request booking' button
+10. Check the Session, Date, ticked slot and Layout shown, then click 'Submit request' and click 'Back to Venue'
+11. In the 'Session' drop-down, choose 'Day 3'
+12. Find 'Orchard Gallery (ORC-GAL)' in the venue list and click its 'Request booking' button
+13. Check the Session, Date, ticked slot and Layout shown, then click 'Submit request' and click 'Back to Venue'
+14. Read the three requests under 'Booking requests'</t>
         </is>
       </c>
     </row>
@@ -1552,7 +1524,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="58" customHeight="1">
+    <row r="4" ht="98.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1560,10 +1532,11 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'Booking Requests' in the sidebar
-2. Find the request for Orchard Seminar Room on 6 Mar 2027
-3. Find the request for Orchard Studio on 2 Mar 2027
-4. Click the event reference on one of them</t>
+          <t>1. Log in as marcus.wong@connectsphere.com / password123
+2. Click 'Booking Requests' in the sidebar
+3. Find the row for Orchard Seminar Room on 6 Mar 2027 and read its Event column
+4. Find the row for Orchard Studio on 2 Mar 2027 and read its Event column
+5. Click the EVT- reference in the 2 Mar row</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1687,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="58" customHeight="1">
+    <row r="4" ht="152.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1722,8 +1695,14 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. As Daniel Tan, open 'SPM42 Town Hall', open the Venue tab and look at its booking requests
-2. Log in as Venue Staff Marcus Wong and click 'Booking Requests' in the sidebar</t>
+          <t>1. Log in as daniel.tan@connectsphere.com / password123
+2. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
+3. Click 'SPM42 Town Hall' in the list
+4. Click the 'Venue' tab
+5. Read the status badge of the request under 'Booking requests'
+6. Log out, then log in as marcus.wong@connectsphere.com / password123
+7. Click 'Booking Requests' in the sidebar
+8. Find the row for SPM42 Town Hall and read every column</t>
         </is>
       </c>
     </row>
@@ -1739,7 +1718,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="71.5" customHeight="1">
+    <row r="6" ht="85" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1748,7 +1727,7 @@
       <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Both screens show the request with the status badge 'Pending'.
-Marcus Wong's list shows venue Orchard Seminar Room, 6 Mar 2027, AM and PM, setup 5 Mar 2027 Night, turnaround 6 Mar 2027 Night, requested by Daniel Tan.</t>
+Marcus Wong's row shows Orchard Seminar Room, '6 Mar 2027 · AM, PM (07:00–18:00)', 'Setup: 5 Mar 2027 Night (19:00–24:00)', 'Turnaround: 6 Mar 2027 Night (19:00–24:00)', and Requested by Daniel Tan.</t>
         </is>
       </c>
     </row>
@@ -1874,7 +1853,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="44.5" customHeight="1">
+    <row r="4" ht="260.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1882,9 +1861,15 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Log in as each account in turn
-2. Open the event 'Town Hall Q4'
-3. Open the Venue tab if it is shown</t>
+          <t>1. Log in as priya.raj@connectsphere.com / password123
+2. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
+3. Click 'Town Hall Q4' in the list
+4. Click the 'Venue' tab
+5. Read the message above the venue list and look for any 'Request booking' button
+6. Log out, log in as rachel.ng@meridianfina.com / password123, click 'My Events', click 'Town Hall Q4' and look for a 'Venue' tab
+7. Log out, log in as grace.lim@connectsphere.com / password123, click 'All Events', click 'Town Hall Q4' and look for a 'Venue' tab
+8. Log out, log in as marcus.wong@connectsphere.com / password123, click 'Booking Requests' and look for any 'Request booking' button
+9. Log out, log in as kenji.sato@connectsphere.com / password123 and look through the sidebar for anywhere to request a venue</t>
         </is>
       </c>
     </row>
@@ -2031,11 +2016,11 @@
       <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Seeded data.
-Logged in as Coordinator Priya Raj (priya.raj@connectsphere.com / password123), assigned to 'Kirana Regional Managers Offsite' (status Under review, 22 Nov 2026 (2026-09-26 + 57) 09:00-17:00).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="31" customHeight="1">
+Logged in as Coordinator Joel Fernandez (joel.fernandez@connectsphere.com / password123), assigned to 'Pearl Delta Supplier Forum' (status Cancelled, 29 Oct 2026 (2026-09-26 + 33) 09:00-14:00).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="98.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2043,8 +2028,11 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Open the event 'Kirana Regional Managers Offsite'
-2. Open the Venue tab (Find a venue)</t>
+          <t>1. Log in as joel.fernandez@connectsphere.com / password123
+2. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
+3. Click 'Pearl Delta Supplier Forum' in the list
+4. Click the 'Venue' tab
+5. Read the message above the venue list and look for any 'Request booking' button</t>
         </is>
       </c>
     </row>
@@ -2056,7 +2044,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Event status: Under review</t>
+          <t>Event status: Cancelled</t>
         </is>
       </c>
     </row>
@@ -2069,7 +2057,7 @@
       <c r="B6" s="13" t="inlineStr">
         <is>
           <t>No 'Request booking' button is shown.
-The page says 'A venue booking can only be requested once the event is Approved or in Planning.'</t>
+The page says 'A venue cannot be requested for a completed, cancelled or rejected event.'</t>
         </is>
       </c>
     </row>
@@ -2182,7 +2170,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="139" customHeight="1">
+    <row r="3" ht="166" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2190,7 +2178,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm42. Seeded data, unchanged:
+          <t>npm run fixtures:spm42 has been run once at the start of this test pass (do not re-run it between cases - later cases use requests made in earlier ones). Seeded data, unchanged:
 - 'Product Showcase' has an Approved booking at Marina Auditorium (MAR-AUD), 21 Oct 2026 (2026-09-26 + 25) 11:00-15:00.
 - 'Pearl Delta Safety Conference' has a Pending booking at Changi Conference Centre (CBP-CONF), 14 Dec 2026 (2026-09-26 + 79) 09:00-17:00.
 - Marina Auditorium is unavailable for maintenance 20-21 Nov 2026 (2026-09-26 + 55 to + 56).
@@ -2198,7 +2186,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="98.5" customHeight="1">
+    <row r="4" ht="382" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2206,12 +2194,22 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Open the event
-2. Open the Venue tab (Find a venue)
-3. Click 'Request booking' on the venue
-4. Tick 'AM (07:00–12:00)' and 'PM (13:00–18:00)' for the date
-5. Click 'Submit request'
-6. Repeat for the next event</t>
+          <t>1. Log in as daniel.tan@connectsphere.com / password123
+2. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
+3. Click 'SPM42 Clash Check' in the list
+4. Click the 'Venue' tab
+5. Find 'Marina Auditorium (MAR-AUD)' in the venue list and click its 'Request booking' button
+6. Make sure 'AM (07:00–12:00)' and 'PM (13:00–18:00)' are ticked for 21 Oct 2026, click 'Submit request' and read the message
+7. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
+8. Click 'Staff Retreat' in the list
+9. Click the 'Venue' tab
+10. Find 'Changi Conference Centre (CBP-CONF)' in the venue list and click its 'Request booking' button
+11. Make sure 'AM (07:00–12:00)' and 'PM (13:00–18:00)' are ticked for 14 Dec 2026, click 'Submit request' and read the message
+12. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
+13. Click 'Sports Meet' in the list
+14. Click the 'Venue' tab
+15. Find 'Marina Auditorium (MAR-AUD)' in the venue list and click its 'Request booking' button
+16. Make sure 'AM (07:00–12:00)' and 'PM (13:00–18:00)' are ticked for 20 Nov 2026, click 'Submit request' and read the message</t>
         </is>
       </c>
     </row>
@@ -2366,7 +2364,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="71.5" customHeight="1">
+    <row r="4" ht="139" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2374,11 +2372,13 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Open the event 'Keynote Rehearsal'
-2. Open the Venue tab (Find a venue)
-3. Click 'Request booking' on 'Marina Auditorium (MAR-AUD)'
-4. Tick only 'PM (13:00–18:00)' for 20 Oct 2026
-5. Click 'Submit request'</t>
+          <t>1. Log in as daniel.tan@connectsphere.com / password123
+2. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
+3. Click 'Keynote Rehearsal' in the list
+4. Click the 'Venue' tab
+5. Find 'Marina Auditorium (MAR-AUD)' in the venue list and click its 'Request booking' button
+6. Make sure only 'PM (13:00–18:00)' is ticked for 20 Oct 2026
+7. Click 'Submit request' and read the message</t>
         </is>
       </c>
     </row>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="139" customHeight="1">
+    <row r="3" ht="166" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2525,14 +2525,14 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm42. It creates:
+          <t>npm run fixtures:spm42 has been run once at the start of this test pass (do not re-run it between cases - later cases use requests made in earlier ones). It creates:
 - 'SPM42 Cancelled Hold' with a Cancelled booking at Orchard Gallery (ORC-GAL), 15 Mar 2027 (2026-09-26 + 170) 09:00-17:00.
 - 'SPM42 Rejected Hold' with a Rejected booking at Marina Auditorium (MAR-AUD), 16 Mar 2027 (2026-09-26 + 171) 09:00-18:00 — had it been approved, its turnaround would hold 16 Mar Night.
 Logged in as Daniel Tan, assigned to the two events in Test data (status Planning, no sessions).</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="98.5" customHeight="1">
+    <row r="4" ht="314.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2540,12 +2540,19 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Open the event
-2. Open the Venue tab (Find a venue)
-3. Click 'Request booking' on the venue
-4. Tick 'AM (07:00–12:00)' and 'PM (13:00–18:00)' for the date
-5. Click 'Submit request'
-6. Repeat for the next event</t>
+          <t>1. Log in as daniel.tan@connectsphere.com / password123
+2. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
+3. Click 'SPM42 After Cancellation' in the list
+4. Click the 'Venue' tab
+5. Find 'Orchard Gallery (ORC-GAL)' in the venue list and click its 'Request booking' button
+6. Make sure 'AM (07:00–12:00)' and 'PM (13:00–18:00)' are ticked for 15 Mar 2027, click 'Submit request' and read the message
+7. Click 'Back to Venue' and read the status under 'Booking requests'
+8. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
+9. Click 'SPM42 After Rejection' in the list
+10. Click the 'Venue' tab
+11. Find 'Marina Auditorium (MAR-AUD)' in the venue list and click its 'Request booking' button
+12. Make sure 'AM (07:00–12:00)' and 'PM (13:00–18:00)' are ticked for 17 Mar 2027, click 'Submit request' and read the message
+13. Click 'Back to Venue' and read the status under 'Booking requests'</t>
         </is>
       </c>
     </row>
@@ -2571,171 +2578,6 @@
       <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Both show 'Booking request sent to Venue Staff.' and the request is Pending.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Sammi Chua</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>46296</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-42-TC17</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="44.5" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>TC04 and TC09 have been run (SPM42 Town Hall and Session 'Day 1' each have a Pending request).
-Logged in as Daniel Tan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="98.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>1. Open the event
-2. Open the Venue tab (Find a venue), choosing the session where there is one
-3. Click 'Request booking' on the venue
-4. Click 'Submit request' with the date and slots already filled in
-5. Repeat for the next attempt</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>1. SPM42 Town Hall, Orchard Studio (ORC-STU), 6 Mar 2027 AM + PM
-2. SPM42 Three-Session Forum, Session 'Day 1', Orchard Gallery (ORC-GAL), 1 Mar 2027 AM</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="85" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>1. 'SPM42 Town Hall already has a venue booking request (Orchard Seminar Room, Pending).'
-2. 'Day 1 already has a venue booking request (Orchard Seminar Room, Pending).'
-No new request is created; Session 'Day 2' and 'Day 3' are unaffected.</t>
         </is>
       </c>
     </row>
@@ -2848,7 +2690,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="98.5" customHeight="1">
+    <row r="3" ht="125.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2856,13 +2698,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm42.
+          <t>npm run fixtures:spm42 has been run once at the start of this test pass (do not re-run it between cases - later cases use requests made in earlier ones).
 Logged in as Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123), assigned to spm42_symposium 'SPM42 Research Symposium' (status Planning, 4 Mar 2027 (2026-09-26 + 159) 09:00-18:00, expects 200, layout Theatre, no sessions).
 Changi Conference Centre (CBP-CONF) has Theatre capacity 260.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="152.5" customHeight="1">
+    <row r="4" ht="260.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2870,14 +2712,18 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Open the event 'SPM42 Research Symposium'
-2. Open the Venue tab (Find a venue)
-3. Find 'Changi Conference Centre (CBP-CONF)' in the results
-4. Click 'Request booking' on it
-5. Tick 'AM (07:00–12:00)' and 'PM (13:00–18:00)' for 4 Mar 2027
-6. Type the text below into 'Venue requirements'
-7. Click 'Submit request'
-8. Log out, log in as Venue Staff Marcus Wong (marcus.wong@connectsphere.com / password123) and click 'Booking Requests' in the sidebar</t>
+          <t>1. Log in as daniel.tan@connectsphere.com / password123
+2. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
+3. Click 'SPM42 Research Symposium' in the list
+4. Click the 'Venue' tab
+5. Find 'Changi Conference Centre (CBP-CONF)' in the venue list and check the badge next to it
+6. Click 'Request booking' on Changi Conference Centre
+7. Check the Date shows 4 Mar 2027 and only 'AM (07:00–12:00)' and 'PM (13:00–18:00)' are ticked
+8. Click in the 'Venue requirements' box and type: Lectern and stage riser at the front; two wireless microphones; doors open 08:30.
+9. Click 'Submit request'
+10. Log out, then log in as marcus.wong@connectsphere.com / password123
+11. Click 'Booking Requests' in the sidebar
+12. Find the row for SPM42 Research Symposium and read its Layout and Requirements</t>
         </is>
       </c>
     </row>
@@ -3021,7 +2867,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="58" customHeight="1">
+    <row r="3" ht="85" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3029,13 +2875,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm42.
+          <t>npm run fixtures:spm42 has been run once at the start of this test pass (do not re-run it between cases - later cases use requests made in earlier ones).
 Logged in as Daniel Tan, assigned to 'SPM42 Research Symposium' (expects 200, Theatre).
 One-North Auditorium (ONE-AUD) has Theatre capacity 180.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="44.5" customHeight="1">
+    <row r="4" ht="112" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -3043,9 +2889,13 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Open the event 'SPM42 Research Symposium'
-2. Open the Venue tab (Find a venue)
-3. Find 'One-North Auditorium (ONE-AUD)' in the results</t>
+          <t>1. Log in as daniel.tan@connectsphere.com / password123
+2. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
+3. Click 'SPM42 Research Symposium' in the list
+4. Click the 'Venue' tab
+5. Find 'One-North Auditorium (ONE-AUD)' in the venue list
+6. Read the badge and the reason shown under it
+7. Look for a 'Request booking' button on it</t>
         </is>
       </c>
     </row>
@@ -3184,7 +3034,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="58" customHeight="1">
+    <row r="3" ht="85" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3192,12 +3042,12 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm42.
+          <t>npm run fixtures:spm42 has been run once at the start of this test pass (do not re-run it between cases - later cases use requests made in earlier ones).
 Logged in as Daniel Tan, assigned to spm42_morning_talk 'SPM42 Morning Talk' (status Planning, 5 Mar 2027 (2026-09-26 + 160) 10:00-12:00, no sessions).</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="98.5" customHeight="1">
+    <row r="4" ht="247" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -3205,12 +3055,18 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Open the event 'SPM42 Morning Talk'
-2. Open the Venue tab (Find a venue)
-3. Click 'Request booking' on 'Orchard Seminar Room (ORC-SEM)'
-4. Tick only 'AM (07:00–12:00)' for 5 Mar 2027
-5. Leave 'Venue requirements' empty
-6. Click 'Submit request'</t>
+          <t>1. Log in as daniel.tan@connectsphere.com / password123
+2. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
+3. Click 'SPM42 Morning Talk' in the list
+4. Click the 'Venue' tab
+5. Find 'Orchard Seminar Room (ORC-SEM)' in the venue list and click its 'Request booking' button
+6. Check the Date shows 5 Mar 2027 and only 'AM (07:00–12:00)' is ticked
+7. Leave the 'Venue requirements' box empty
+8. Click 'Submit request'
+9. Click 'Back to Venue' and read the request under 'Booking requests'
+10. Log out, then log in as marcus.wong@connectsphere.com / password123
+11. Click 'Booking Requests' in the sidebar
+12. Find the row for SPM42 Morning Talk and read its Requirements</t>
         </is>
       </c>
     </row>
@@ -3228,7 +3084,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="58" customHeight="1">
+    <row r="6" ht="85" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3237,7 +3093,8 @@
       <c r="B6" s="13" t="inlineStr">
         <is>
           <t>'Booking request sent to Venue Staff.' is shown.
-The request shows 5 Mar 2027, AM (07:00–12:00) — the whole slot, not the event's own 10:00–12:00 — and Requirements 'None given'.</t>
+Under 'Booking requests' the request reads '5 Mar 2027 · AM (07:00–12:00)' — the whole slot, not the event's own 10:00–12:00.
+Marcus Wong's Booking Requests row shows Requirements 'None given'.</t>
         </is>
       </c>
     </row>
@@ -3350,7 +3207,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="58" customHeight="1">
+    <row r="3" ht="85" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3358,12 +3215,12 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm42.
+          <t>npm run fixtures:spm42 has been run once at the start of this test pass (do not re-run it between cases - later cases use requests made in earlier ones).
 Logged in as Daniel Tan, assigned to spm42_town_hall 'SPM42 Town Hall' (status Planning, 6 Mar 2027 (2026-09-26 + 161) 09:00-17:00, no sessions).</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="85" customHeight="1">
+    <row r="4" ht="193" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -3371,11 +3228,15 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Open the event 'SPM42 Town Hall'
-2. Open the Venue tab (Find a venue)
-3. Click 'Request booking' on 'Orchard Seminar Room (ORC-SEM)'
-4. Check the date and slots already filled in
-5. Click 'Submit request'</t>
+          <t>1. Log in as daniel.tan@connectsphere.com / password123
+2. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
+3. Click 'SPM42 Town Hall' in the list
+4. Click the 'Venue' tab
+5. Check there is no 'Session' drop-down above the venue list
+6. Find 'Orchard Seminar Room (ORC-SEM)' in the venue list and click its 'Request booking' button
+7. Check the Date shows 6 Mar 2027 and 'AM (07:00–12:00)' and 'PM (13:00–18:00)' are already ticked
+8. Click 'Submit request'
+9. Click 'Back to Venue' and read the request under 'Booking requests'</t>
         </is>
       </c>
     </row>
@@ -3393,7 +3254,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="58" customHeight="1">
+    <row r="6" ht="71.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3401,9 +3262,9 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>No Session field is shown. The date is 6 Mar 2027 with AM and PM already ticked (the event's own time).
+          <t>No Session drop-down is shown. The Date is 6 Mar 2027 with AM and PM already ticked (the event's own time).
 'Booking request sent to Venue Staff.' is shown.
-The request shows 6 Mar 2027, AM and PM, 07:00–18:00.</t>
+Under 'Booking requests' the request reads '6 Mar 2027 · AM, PM (07:00–18:00)'.</t>
         </is>
       </c>
     </row>
@@ -3516,7 +3377,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="85" customHeight="1">
+    <row r="3" ht="112" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3524,13 +3385,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm42.
+          <t>npm run fixtures:spm42 has been run once at the start of this test pass (do not re-run it between cases - later cases use requests made in earlier ones).
 Logged in as Daniel Tan, assigned to spm42_refusals 'SPM42 Refusal Checks' (status Planning, 7 Mar 2027 (2026-09-26 + 162) 09:00-17:00, no sessions).
 Booking request screen open for it at 'Orchard Seminar Room (ORC-SEM)'.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="71.5" customHeight="1">
+    <row r="4" ht="206.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -3538,10 +3399,16 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Untick every slot
-2. Click 'Submit request'
-3. Tick 'AM (07:00–12:00)' and 'Night (19:00–24:00)', leave PM unticked
-4. Click 'Submit request'</t>
+          <t>1. Log in as daniel.tan@connectsphere.com / password123
+2. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
+3. Click 'SPM42 Refusal Checks' in the list
+4. Click the 'Venue' tab
+5. Find 'Orchard Seminar Room (ORC-SEM)' in the venue list and click its 'Request booking' button
+6. Untick 'AM (07:00–12:00)' and 'PM (13:00–18:00)' so no slot is ticked
+7. Click 'Submit request' and read the message
+8. Tick 'AM (07:00–12:00)' and 'Night (19:00–24:00)'; leave 'PM (13:00–18:00)' unticked
+9. Click 'Submit request' and read the message
+10. Click 'Cancel' and check 'Booking requests' on the Venue tab</t>
         </is>
       </c>
     </row>
@@ -3682,7 +3549,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="85" customHeight="1">
+    <row r="3" ht="112" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3690,13 +3557,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm42.
+          <t>npm run fixtures:spm42 has been run once at the start of this test pass (do not re-run it between cases - later cases use requests made in earlier ones).
 Logged in as Daniel Tan, assigned to the three events in Test data (all status Planning, no sessions).
 Orchard Seminar Room (ORC-SEM): setup 60 min, teardown 30 min. Changi Conference Centre (CBP-CONF): setup 120 min, teardown 90 min.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="98.5" customHeight="1">
+    <row r="4" ht="382" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -3704,13 +3571,22 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Open the event
-2. Open the Venue tab (Find a venue)
-3. Click 'Request booking' on the venue
-4. Tick the slots for the date
-5. Read the setup and turnaround lines
-6. Click 'Submit request'
-7. Repeat for the next event</t>
+          <t>1. Log in as daniel.tan@connectsphere.com / password123
+2. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
+3. Click 'SPM42 Early Briefing' in the list
+4. Click the 'Venue' tab
+5. Find 'Orchard Seminar Room (ORC-SEM)' in the venue list and click its 'Request booking' button
+6. Check only 'AM (07:00–12:00)' is ticked for 8 Mar 2027, read the 'Setup:' and 'Turnaround:' lines, then click 'Submit request'
+7. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
+8. Click 'SPM42 Late Show' in the list
+9. Click the 'Venue' tab
+10. Find 'Orchard Seminar Room (ORC-SEM)' in the venue list and click its 'Request booking' button
+11. Check only 'Night (19:00–24:00)' is ticked for 9 Mar 2027, read the 'Setup:' and 'Turnaround:' lines, then click 'Submit request'
+12. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
+13. Click 'SPM42 Networking Evening' in the list
+14. Click the 'Venue' tab
+15. Find 'Changi Conference Centre (CBP-CONF)' in the venue list and click its 'Request booking' button
+16. Check only 'PM (13:00–18:00)' and 'Night (19:00–24:00)' are ticked for 11 Mar 2027, read the 'Setup:' and 'Turnaround:' lines, then click 'Submit request'</t>
         </is>
       </c>
     </row>
@@ -3852,7 +3728,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="85" customHeight="1">
+    <row r="3" ht="112" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3860,13 +3736,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm42.
+          <t>npm run fixtures:spm42 has been run once at the start of this test pass (do not re-run it between cases - later cases use requests made in earlier ones).
 Logged in as Daniel Tan, assigned to spm42_plain_pm 'SPM42 Plain Afternoon' (status Planning, 10 Mar 2027 (2026-09-26 + 165) 14:00-17:00, expects 30, Classroom, no sessions).
 Fixture venue 'SPM42 Plain Room' (SPM42-PLN) has setup 0 min and teardown 0 min.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="85" customHeight="1">
+    <row r="4" ht="193" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -3874,11 +3750,16 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Open the event 'SPM42 Plain Afternoon'
-2. Open the Venue tab (Find a venue)
-3. Click 'Request booking' on 'SPM42 Plain Room (SPM42-PLN)'
-4. Tick 'PM (13:00–18:00)' and 'Night (19:00–24:00)' for 10 Mar 2027
-5. Click 'Submit request'</t>
+          <t>1. Log in as daniel.tan@connectsphere.com / password123
+2. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
+3. Click 'SPM42 Plain Afternoon' in the list
+4. Click the 'Venue' tab
+5. Find 'SPM42 Plain Room (SPM42-PLN)' in the venue list and click its 'Request booking' button
+6. Read the line under the slots
+7. Tick 'Night (19:00–24:00)' as well, so 'PM (13:00–18:00)' and 'Night (19:00–24:00)' are both ticked for 10 Mar 2027
+8. Check the line under the slots has not changed
+9. Click 'Submit request'
+10. Click 'Back to Venue' and read the request under 'Booking requests'</t>
         </is>
       </c>
     </row>
@@ -3904,9 +3785,9 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The screen shows 'No setup or turnaround needed at this venue.'
+          <t>Before and after ticking Night, the line under the slots reads 'No setup or turnaround needed at this venue.'
 'Booking request sent to Venue Staff.' is shown.
-The request holds 10 Mar 2027 PM and Night — nothing before or after.</t>
+Under 'Booking requests' the request reads '10 Mar 2027 · PM, Night (13:00–24:00)' — nothing before or after.</t>
         </is>
       </c>
     </row>
@@ -4019,7 +3900,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="71.5" customHeight="1">
+    <row r="3" ht="112" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -4027,12 +3908,12 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm42 (so Day 2 has no request yet).
+          <t>npm run fixtures:spm42 has been run once at the start of this test pass (do not re-run it between cases - later cases use requests made in earlier ones). Run this case before TC09, so Day 2 has no request yet.
 Logged in as Daniel Tan, assigned to spm42_three_sessions 'SPM42 Three-Session Forum' (Day 2: 2 Mar 2027 (2026-09-26 + 157) 14:00-17:00) and to 'SPM42 Refusal Checks' (7 Mar 2027 09:00-17:00, no sessions).</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="152.5" customHeight="1">
+    <row r="4" ht="287.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -4040,11 +3921,19 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Open 'SPM42 Three-Session Forum', open the Venue tab, choose Session 'Day 2' and click 'Request booking' on 'Orchard Studio (ORC-STU)'
-2. Tick only 'AM (07:00–12:00)' for 2 Mar 2027 and click 'Submit request'
-3. Change the date to 1 Mar 2027, tick only 'PM (13:00–18:00)' and click 'Submit request'
-4. Open 'SPM42 Refusal Checks', open the Venue tab and click 'Request booking' on 'Orchard Seminar Room (ORC-SEM)'
-5. Tick only 'AM (07:00–12:00)' for 7 Mar 2027 and click 'Submit request'</t>
+          <t>1. Log in as daniel.tan@connectsphere.com / password123
+2. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
+3. Click 'SPM42 Three-Session Forum' in the list
+4. Click the 'Venue' tab
+5. In the 'Session' drop-down, choose 'Day 2'
+6. Find 'Orchard Studio (ORC-STU)' in the venue list and click its 'Request booking' button
+7. Untick 'PM (13:00–18:00)', tick only 'AM (07:00–12:00)', then click 'Submit request' and read the message
+8. Change the Date to 1 Mar 2027, tick only 'PM (13:00–18:00)', then click 'Submit request' and read the message
+9. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
+10. Click 'SPM42 Refusal Checks' in the list
+11. Click the 'Venue' tab
+12. Find 'Orchard Seminar Room (ORC-SEM)' in the venue list and click its 'Request booking' button
+13. Untick 'PM (13:00–18:00)' so only 'AM (07:00–12:00)' is ticked for 7 Mar 2027, then click 'Submit request' and read the message</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SPM-59: Mark the three cases quoting the old closed-event message Updated
SPM-59 made the messages that refuse an action on a closed event name
withdrawn events. SPM-42-TC13, SPM-43-TC06 and SPM-54-TC13 quote the old
wording; per docs/test-cases/README.md this PR updates them instead of
leaving a Known Gap, as SPM-80 did in fb8eb36:

- Workbooks: Status Updated, Change # #103 (TC06: "#128 (Week 7 #1); #103"),
  and a v2 note in row 1 (TC06 already had v2, so v3). Edited in place; no
  execution block changed.
- DECOMMISSIONED.md: one row each; Updated total 106 -> 109.
- CHANGES.md: new "Forum #103 - Record request withdrawal" entry.
- DOCUMENTATION.md: Known Gaps row removed; noted in the SPM-59 entry.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-42_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-42_Test_Cases.xlsx
@@ -34,7 +34,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -82,6 +82,10 @@
     </font>
     <font>
       <color rgb="FF000000"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="5">
@@ -195,7 +199,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -239,6 +243,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1162,11 +1169,15 @@
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="H16" s="14" t="n"/>
-      <c r="I16" s="14" t="n"/>
+      <c r="I16" s="14" t="inlineStr">
+        <is>
+          <t>#103</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="25.05" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
@@ -1301,8 +1312,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21"/>
     <row r="22" ht="13.05" customHeight="1">
       <c r="A22" s="17" t="inlineStr">
         <is>
@@ -1502,7 +1511,6 @@
       </c>
       <c r="F30" s="16" t="n"/>
     </row>
-    <row r="31"/>
     <row r="32" ht="166.05" customHeight="1">
       <c r="A32" s="17" t="inlineStr">
         <is>
@@ -5233,53 +5241,61 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.59765625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.796875" customWidth="1" min="1" max="1"/>
     <col width="56.796875" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13.05" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="64" customHeight="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>v2 (2026-10-23): The page now reads 'A venue cannot be requested for a completed, cancelled, rejected or withdrawn event.' instead of 'A venue cannot be requested for a completed, cancelled or rejected event.' (SPM-59, discussion #103: the messages that refuse an action on a closed event now name withdrawn events too). Read the expected result with the new wording. The behaviour this case checks is unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="13.05" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.55" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="B2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="17.55" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>SPM-42-TC13</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="71.55" customHeight="1">
-      <c r="A3" s="10" t="inlineStr">
+    <row r="4" ht="71.55" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Seeded data.
 Logged in as Coordinator Joel Fernandez (joel.fernandez@connectsphere.com / password123), assigned to 'Pearl Delta Supplier Forum' (status Cancelled, 29 Oct 2026 (2026-09-26 + 33) 09:00-14:00).</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="98.55" customHeight="1">
-      <c r="A4" s="10" t="inlineStr">
+    <row r="5" ht="98.55" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>1. Log in as joel.fernandez@connectsphere.com / password123
 2. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
@@ -5289,188 +5305,193 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="17.55" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
+    <row r="6" ht="17.55" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Event status: Cancelled</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="44.55" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
+    <row r="7" ht="44.55" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>No 'Request booking' button is shown.
 The page says 'A venue cannot be requested for a completed, cancelled or rejected event.'</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="17.55" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
+    <row r="8" ht="17.55" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Sammi Chua</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="12.5" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
+    <row r="9" ht="12.5" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B8" s="12" t="n">
+      <c r="B9" s="12" t="n">
         <v>46296</v>
       </c>
     </row>
-    <row r="10" ht="13.05" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="10"/>
+    <row r="11" ht="13.05" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11" ht="37.5" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12" ht="37.5" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>No 'Request booking' button is shown.
 The page says 'A venue cannot be requested for a completed, cancelled or rejected event.'</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="12.5" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="14" ht="12.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Executed by</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Sammi</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="12.5" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="12" t="n">
+      <c r="B16" s="12" t="n">
         <v>46296</v>
       </c>
     </row>
-    <row r="17" ht="13.05" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="17"/>
+    <row r="18" ht="13.05" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n"/>
-    </row>
-    <row r="18" ht="58.05" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="B18" s="5" t="n"/>
+    </row>
+    <row r="19" ht="58.05" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>On the cancelled event's Venue tab the page read 'A venue cannot be requested for a completed, cancelled or rejected event.' and no Request booking button was present on any venue card.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="17.55" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B19" s="13" t="inlineStr">
-        <is>
-          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="20" ht="17.55" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>NA</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="21" ht="17.55" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="17.55" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">TAN JORDAN </t>
         </is>
       </c>
     </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B22" s="12" t="n">
+      <c r="B23" s="12" t="n">
         <v>46296</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Revert "Spm 59 record request withdrawal"
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-42_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-42_Test_Cases.xlsx
@@ -34,7 +34,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -82,10 +82,6 @@
     </font>
     <font>
       <color rgb="FF000000"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="5">
@@ -199,7 +195,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -243,9 +239,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1169,15 +1162,11 @@
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H16" s="14" t="n"/>
-      <c r="I16" s="14" t="inlineStr">
-        <is>
-          <t>#103</t>
-        </is>
-      </c>
+      <c r="I16" s="14" t="n"/>
     </row>
     <row r="17" ht="25.05" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
@@ -1312,6 +1301,8 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
+    <row r="21"/>
     <row r="22" ht="13.05" customHeight="1">
       <c r="A22" s="17" t="inlineStr">
         <is>
@@ -1511,6 +1502,7 @@
       </c>
       <c r="F30" s="16" t="n"/>
     </row>
+    <row r="31"/>
     <row r="32" ht="166.05" customHeight="1">
       <c r="A32" s="17" t="inlineStr">
         <is>
@@ -5241,61 +5233,53 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.59765625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.796875" customWidth="1" min="1" max="1"/>
     <col width="56.796875" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="64" customHeight="1">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>v2 (2026-10-23): The page now reads 'A venue cannot be requested for a completed, cancelled, rejected or withdrawn event.' instead of 'A venue cannot be requested for a completed, cancelled or rejected event.' (SPM-59, discussion #103: the messages that refuse an action on a closed event now name withdrawn events too). Read the expected result with the new wording. The behaviour this case checks is unchanged.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="13.05" customHeight="1">
-      <c r="A2" s="1" t="inlineStr">
+    <row r="1" ht="13.05" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-    </row>
-    <row r="3" ht="17.55" customHeight="1">
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.55" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>SPM-42-TC13</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="71.55" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>Test Case ID</t>
+          <t>Pre-conditions</t>
         </is>
       </c>
       <c r="B3" s="11" t="inlineStr">
-        <is>
-          <t>SPM-42-TC13</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="71.55" customHeight="1">
-      <c r="A4" s="10" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Seeded data.
 Logged in as Coordinator Joel Fernandez (joel.fernandez@connectsphere.com / password123), assigned to 'Pearl Delta Supplier Forum' (status Cancelled, 29 Oct 2026 (2026-09-26 + 33) 09:00-14:00).</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="98.55" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
+    <row r="4" ht="98.55" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>1. Log in as joel.fernandez@connectsphere.com / password123
 2. Click 'All Events' in the sidebar (the list has no search box - use Ctrl+F to find the event)
@@ -5305,193 +5289,188 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="17.55" customHeight="1">
+    <row r="5" ht="17.55" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Event status: Cancelled</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.55" customHeight="1">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>Test Data</t>
+          <t>Expected Result</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>Event status: Cancelled</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="44.55" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>No 'Request booking' button is shown.
 The page says 'A venue cannot be requested for a completed, cancelled or rejected event.'</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="17.55" customHeight="1">
+    <row r="7" ht="17.55" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="12.5" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>Sammi Chua</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="12.5" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B9" s="12" t="n">
+      <c r="B8" s="12" t="n">
         <v>46296</v>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11" ht="13.05" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="10" ht="13.05" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="6" t="n"/>
-    </row>
-    <row r="12" ht="37.5" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="6" t="n"/>
+    </row>
+    <row r="11" ht="37.5" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>No 'Request booking' button is shown.
 The page says 'A venue cannot be requested for a completed, cancelled or rejected event.'</t>
         </is>
       </c>
     </row>
+    <row r="12" ht="12.5" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="14" ht="12.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Executed by</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Sammi</t>
         </is>
       </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Sammi</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="12.5" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="12" t="n">
+      <c r="B15" s="12" t="n">
         <v>46296</v>
       </c>
     </row>
-    <row r="17"/>
-    <row r="18" ht="13.05" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="17" ht="13.05" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n"/>
-    </row>
-    <row r="19" ht="58.05" customHeight="1">
+      <c r="B17" s="5" t="n"/>
+    </row>
+    <row r="18" ht="58.05" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>On the cancelled event's Venue tab the page read 'A venue cannot be requested for a completed, cancelled or rejected event.' and no Request booking button was present on any venue card.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="17.55" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>On the cancelled event's Venue tab the page read 'A venue cannot be requested for a completed, cancelled or rejected event.' and no Request booking button was present on any venue card.</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="20" ht="17.55" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B20" s="13" t="inlineStr">
-        <is>
-          <t>Pass</t>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="21" ht="17.55" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Executed by</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="17.55" customHeight="1">
+          <t xml:space="preserve">TAN JORDAN </t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAN JORDAN </t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B23" s="12" t="n">
+      <c r="B22" s="12" t="n">
         <v>46296</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>